<commit_message>
Commit vor PCB Layout
</commit_message>
<xml_diff>
--- a/Bauteile/Pinlayout_Microcontroller.xlsx
+++ b/Bauteile/Pinlayout_Microcontroller.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Semester6\Projektarbeit\Joystick_STM_3_3V\Bauteile\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Semester6\Projektarbeit\Projektarbeit_Joystick\Bauteile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5457AF5C-F399-4D2B-A849-ABF77B488AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ECA1DB5-F7FF-44D9-BA7B-690DBAF88768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BF97E7C2-419E-42F4-87E5-5936AB5A7FBA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BF97E7C2-419E-42F4-87E5-5936AB5A7FBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="81">
   <si>
     <t>Pin Nr.</t>
   </si>
@@ -260,6 +260,9 @@
   </si>
   <si>
     <t>Vtref_3.3V</t>
+  </si>
+  <si>
+    <t>Implementiert</t>
   </si>
 </sst>
 </file>
@@ -274,7 +277,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -311,6 +314,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -339,9 +348,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -350,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -365,6 +372,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -404,16 +415,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>19903</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>714668</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>283882</xdr:rowOff>
+      <xdr:rowOff>276411</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>105868</xdr:colOff>
+      <xdr:colOff>38633</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>83379</xdr:rowOff>
+      <xdr:rowOff>75908</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -436,7 +447,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7572668" y="470647"/>
+          <a:off x="8708197" y="463176"/>
           <a:ext cx="4657965" cy="3900850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -766,15 +777,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B684EB25-46FB-4AFF-8E98-4363EF5EDC4B}">
-  <dimension ref="B2:G31"/>
+  <dimension ref="B2:H31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.90625" customWidth="1"/>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="96.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" ht="29" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -790,8 +803,11 @@
       <c r="F2" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H2" s="10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3">
         <v>25</v>
       </c>
@@ -801,7 +817,7 @@
       <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="13" t="s">
         <v>8</v>
       </c>
       <c r="F3" s="4" t="s">
@@ -810,8 +826,9 @@
       <c r="G3" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="H3" s="11"/>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" s="3">
         <v>24</v>
       </c>
@@ -821,12 +838,13 @@
       <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="13"/>
       <c r="F4" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" s="3">
         <v>22</v>
       </c>
@@ -836,12 +854,13 @@
       <c r="D5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="11"/>
+      <c r="E5" s="13"/>
       <c r="F5" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
         <v>23</v>
       </c>
@@ -851,12 +870,13 @@
       <c r="D6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="11"/>
+      <c r="E6" s="13"/>
       <c r="F6" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="H6" s="11"/>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="5">
         <v>30</v>
       </c>
@@ -866,7 +886,7 @@
       <c r="D7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="14" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="4" t="s">
@@ -875,8 +895,9 @@
       <c r="G7" s="9" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" s="5">
         <v>29</v>
       </c>
@@ -886,12 +907,13 @@
       <c r="D8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="12"/>
+      <c r="E8" s="14"/>
       <c r="F8" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="5">
         <v>27</v>
       </c>
@@ -901,12 +923,13 @@
       <c r="D9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="12"/>
+      <c r="E9" s="14"/>
       <c r="F9" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" s="5">
         <v>28</v>
       </c>
@@ -916,12 +939,13 @@
       <c r="D10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="12"/>
+      <c r="E10" s="14"/>
       <c r="F10" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="H10" s="11"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="6">
         <v>33</v>
       </c>
@@ -931,7 +955,7 @@
       <c r="D11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="15" t="s">
         <v>19</v>
       </c>
       <c r="F11" s="4" t="s">
@@ -941,7 +965,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" s="6">
         <v>35</v>
       </c>
@@ -951,12 +975,12 @@
       <c r="D12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="13"/>
+      <c r="E12" s="15"/>
       <c r="F12" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B13" s="6">
         <v>36</v>
       </c>
@@ -966,12 +990,12 @@
       <c r="D13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E13" s="13"/>
+      <c r="E13" s="15"/>
       <c r="F13" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B14" s="6">
         <v>34</v>
       </c>
@@ -981,12 +1005,12 @@
       <c r="D14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="13"/>
+      <c r="E14" s="15"/>
       <c r="F14" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" s="6">
         <v>37</v>
       </c>
@@ -996,12 +1020,12 @@
       <c r="D15" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E15" s="13"/>
+      <c r="E15" s="15"/>
       <c r="F15" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" s="7"/>
       <c r="C16" s="7" t="s">
         <v>21</v>
@@ -1009,13 +1033,13 @@
       <c r="D16" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E16" s="16" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="G16" s="12" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1027,11 +1051,11 @@
       <c r="D17" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="14"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G17" s="10"/>
+      <c r="G17" s="12"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" s="7">
@@ -1043,11 +1067,11 @@
       <c r="D18" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="15"/>
+      <c r="E18" s="17"/>
       <c r="F18" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G18" s="10"/>
+      <c r="G18" s="12"/>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B19" s="7">
@@ -1059,11 +1083,11 @@
       <c r="D19" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E19" s="15"/>
+      <c r="E19" s="17"/>
       <c r="F19" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G19" s="10"/>
+      <c r="G19" s="12"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B20" s="7">
@@ -1075,11 +1099,11 @@
       <c r="D20" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="15"/>
+      <c r="E20" s="17"/>
       <c r="F20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G20" s="10"/>
+      <c r="G20" s="12"/>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B21" s="7">
@@ -1091,11 +1115,11 @@
       <c r="D21" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="15"/>
+      <c r="E21" s="17"/>
       <c r="F21" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G21" s="10"/>
+      <c r="G21" s="12"/>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B22" s="7">
@@ -1107,11 +1131,11 @@
       <c r="D22" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="15"/>
+      <c r="E22" s="17"/>
       <c r="F22" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G22" s="10"/>
+      <c r="G22" s="12"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B23" s="7"/>
@@ -1121,11 +1145,11 @@
       <c r="D23" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E23" s="15"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="G23" s="10"/>
+      <c r="G23" s="12"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24" s="7"/>
@@ -1135,11 +1159,11 @@
       <c r="D24" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="15"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G24" s="10"/>
+      <c r="G24" s="12"/>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B25" s="7"/>
@@ -1147,11 +1171,11 @@
       <c r="D25" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E25" s="15"/>
+      <c r="E25" s="17"/>
       <c r="F25" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G25" s="10"/>
+      <c r="G25" s="12"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B26" s="8">

</xml_diff>